<commit_message>
feat: Add CustomTkinter Desktop GUI, 1-Click Launchers, Mobile Colab Runner, and Showcase Website
</commit_message>
<xml_diff>
--- a/data_folder/jobs_template.xlsx
+++ b/data_folder/jobs_template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Jobs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Jobs_To_Apply" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,17 +419,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Job Title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Company Name</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Job Link (Direct ATS or Portal)</t>
+          <t>Job URL</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -439,24 +439,24 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Solace</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155195-senior-full-stack-engineer-7</t>
+          <t>https://boards.greenhouse.io/stripe/jobs/example</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -466,24 +466,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Target Role</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Software Engineer, Customer Platform</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Samsara</t>
+          <t>Frontend Developer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154343-senior-software-engineer-agentic-customer-platform-poland-remote-b2b</t>
+          <t>https://jobs.lever.co/figma/example</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -493,24 +493,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ATS Greenhouse</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Product Engineer</t>
+          <t>Vercel</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Help Scout</t>
+          <t>Full Stack Engineer</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153199-mid-sr-product-engineer-intelligence</t>
+          <t>https://jobs.ashbyhq.com/vercel/example</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -520,7 +520,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ATS Lever</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>